<commit_message>
feat(registers): new POL/PRO-style header — logo strip + navy banner + merged value cells
</commit_message>
<xml_diff>
--- a/public/ims/REG-02-Lead-Register.xlsx
+++ b/public/ims/REG-02-Lead-Register.xlsx
@@ -11,7 +11,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
+  <si>
+    <t>Marketing &amp; Lead Generation  —  Confidential — Internal Use Only</t>
+  </si>
+  <si>
+    <t>PREQAL INTEGRATED MANAGEMENT SYSTEM  •  Controlled Document — Internal Use Only</t>
+  </si>
   <si>
     <t>TITLE</t>
   </si>
@@ -19,40 +25,28 @@
     <t>PREQAL LEAD REGISTER</t>
   </si>
   <si>
-    <t>INVITED</t>
-  </si>
-  <si>
-    <t>CREATED</t>
-  </si>
-  <si>
-    <t>REVISED</t>
-  </si>
-  <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
     <t>DCN</t>
   </si>
   <si>
     <t>PQL-REG-02</t>
   </si>
   <si>
+    <t>SCOPE</t>
+  </si>
+  <si>
+    <t>COMMERCIAL — LEAD CAPTURE TO QUALIFIED</t>
+  </si>
+  <si>
+    <t>CREATION DATE</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>APPROVAL DATE</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>SCOPE</t>
-  </si>
-  <si>
-    <t>COMMERCIAL — LEAD CAPTURE TO QUALIFIED</t>
-  </si>
-  <si>
-    <t>CREATION DATE</t>
-  </si>
-  <si>
-    <t>2026-05-14</t>
-  </si>
-  <si>
-    <t>APPROVAL DATE</t>
   </si>
   <si>
     <t>VERSION NUMBER</t>
@@ -137,10 +131,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-  </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -149,42 +140,18 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="36"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF334155"/>
       <sz val="9"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="18"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -202,6 +169,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
@@ -213,11 +185,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFBEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -253,38 +220,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -309,11 +267,11 @@
   <xdr:oneCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>16000</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>71999</xdr:rowOff>
+      <xdr:colOff>96000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>20000</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="857250" cy="952500"/>
+    <xdr:ext cx="209550" cy="228600"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -329,6 +287,45 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>256000</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>71999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="857250" cy="952500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -670,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -684,326 +681,339 @@
     <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="5">
-        <v>3</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="7">
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="7">
-        <v>0</v>
-      </c>
-      <c r="J3" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="H6" s="8">
-        <v>1</v>
-      </c>
-      <c r="I6" s="8">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-    </row>
-    <row r="10" ht="6" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="C10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" ht="6" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="D13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="E13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="F13" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="G13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="H13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="I13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="J13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="K13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J12" s="10" t="s">
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="C14" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="D14" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="E14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="F14" s="8">
+        <v>0</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="K14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="11">
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="9">
         <v>0</v>
       </c>
-      <c r="G13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="K13" s="11" t="s">
+      <c r="G15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K15" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="16" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="E16" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="F16" s="8">
+        <v>0</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="12">
-        <v>0</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="K14" s="12" t="s">
+      <c r="K16" s="8" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="11">
-        <v>0</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A2:B10"/>
-    <mergeCell ref="E2:E9"/>
-    <mergeCell ref="H3:H5"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="I6:I9"/>
-    <mergeCell ref="J6:J9"/>
+  <mergeCells count="11">
+    <mergeCell ref="B1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:B10"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="D4:K4"/>
+    <mergeCell ref="D5:K5"/>
+    <mergeCell ref="D6:K6"/>
+    <mergeCell ref="D7:K7"/>
+    <mergeCell ref="D8:K8"/>
+    <mergeCell ref="D9:K9"/>
+    <mergeCell ref="D10:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>